<commit_message>
nmv 22 07 2026
</commit_message>
<xml_diff>
--- a/TS Jatai Working/Padam Input Templates/TS 3.4 Padam Input Template.xlsx
+++ b/TS Jatai Working/Padam Input Templates/TS 3.4 Padam Input Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ALL IMP DATA\GitHub\texts\TS Jatai Working\Padam Input Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8C4DDD-E188-4DAE-A8DF-955E31310D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83FD1C9E-B563-448A-806B-7189B8E0CD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8562" uniqueCount="1618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8570" uniqueCount="1619">
   <si>
     <t>PS</t>
   </si>
@@ -5014,6 +5014,9 @@
   </si>
   <si>
     <t>saqmarddhu#kaqmiti# saM - arddhu#kam</t>
+  </si>
+  <si>
+    <t>anu#matiqrityanu# - maqtiqH</t>
   </si>
 </sst>
 </file>
@@ -67377,8 +67380,8 @@
       <c r="O1779" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="V1779" s="36" t="s">
-        <v>1382</v>
+      <c r="V1779" s="37" t="s">
+        <v>1618</v>
       </c>
     </row>
     <row r="1780" spans="9:22" ht="20.25" x14ac:dyDescent="0.25">

</xml_diff>